<commit_message>
Add deeper Adeseun source research
</commit_message>
<xml_diff>
--- a/outputs/adeseun-wikipedia-dossier-2026-10-05/adeseun-oyeneye-wikipedia-fact-dossier.xlsx
+++ b/outputs/adeseun-wikipedia-dossier-2026-10-05/adeseun-oyeneye-wikipedia-fact-dossier.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc6ba0e7455ea463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fact dossier" sheetId="2" r:id="Re656cc400dee4b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rc8b952e4dce4465d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books" sheetId="4" r:id="R4ce4798d2dec4b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site claim conflicts" sheetId="5" r:id="R9feb9279d6f34072"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gaps &amp; actions" sheetId="6" r:id="Rf5240369d4a84829"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wikipedia plan" sheetId="7" r:id="R718a5910835149d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R40eac25ee0dc4d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fact dossier" sheetId="2" r:id="R0cda55271e1c457d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rb1ff148aaf3d44f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books" sheetId="4" r:id="R44dc44f554a44683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site claim conflicts" sheetId="5" r:id="Rc107dc4050f64ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gaps &amp; actions" sheetId="6" r:id="Rac469bbc5527432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wikipedia plan" sheetId="7" r:id="Rf335ca6b76304431"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -233,7 +233,7 @@
         <x:color rgb="FF0B6B2B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE3F8E8"/>
         </x:patternFill>
       </x:fill>
@@ -244,7 +244,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -255,7 +255,7 @@
         <x:color rgb="FF8A1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -265,7 +265,7 @@
         <x:color rgb="FF1F2933"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4D6"/>
         </x:patternFill>
       </x:fill>
@@ -275,8 +275,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FactDossierTable" displayName="FactDossierTable" ref="A4:K30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:K30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FactDossierTable" displayName="FactDossierTable" ref="A4:K38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:K38"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Category"/>
@@ -295,8 +295,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SourcesTable" displayName="SourcesTable" ref="A4:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L22"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SourcesTable" displayName="SourcesTable" ref="A4:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L31"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -352,8 +352,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GapsTable" displayName="GapsTable" ref="A4:H12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:H12"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GapsTable" displayName="GapsTable" ref="A4:H14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:H14"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Gap"/>
@@ -621,7 +621,7 @@
         <x:v>Reason</x:v>
       </x:c>
       <x:c r="B4" s="28" t="str">
-        <x:v>The source set verifies many facts, but independent significant biographical coverage is still thin.</x:v>
+        <x:v>Deeper search found more independent direct mentions, but not yet the profile-depth coverage needed for a defensible standalone biography.</x:v>
       </x:c>
       <x:c r="C4" s="28" t="str"/>
       <x:c r="D4" s="28" t="str"/>
@@ -651,7 +651,7 @@
       <x:c r="B6" s="9" t="str"/>
       <x:c r="C6" s="9" t="n">
         <x:f>COUNTA('Fact dossier'!A5:A200)</x:f>
-        <x:v>26</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
         <x:v>Evidence inventory size</x:v>
@@ -667,7 +667,7 @@
       <x:c r="B7" s="9" t="str"/>
       <x:c r="C7" s="9" t="n">
         <x:f>COUNTIF('Fact dossier'!F5:F200,"Verified")+COUNTIF('Fact dossier'!F5:F200,"Partially verified")+COUNTIF('Fact dossier'!F5:F200,"Verified for event only")</x:f>
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
         <x:v>Shows how much is usable for a draft</x:v>
@@ -683,7 +683,7 @@
       <x:c r="B8" s="9" t="str"/>
       <x:c r="C8" s="9" t="n">
         <x:f>COUNTIF(Sources!G5:G100,"Independent")</x:f>
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>Not all independent rows are significant biography coverage</x:v>
@@ -715,7 +715,7 @@
       <x:c r="B10" s="9" t="str"/>
       <x:c r="C10" s="9" t="n">
         <x:f>COUNTIFS('Gaps &amp; actions'!G5:G100,"High",'Gaps &amp; actions'!H5:H100,"Open")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>Core work remaining before AfC</x:v>
@@ -729,14 +729,14 @@
         <x:v>Recommendation</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Build a draft only after stronger independent coverage is found.</x:v>
-      </x:c>
-      <x:c r="C11" s="10" t="str"/>
+        <x:v>Keep building the source dossier before drafting a full article.</x:v>
+      </x:c>
+      <x:c r="C11" s="10"/>
       <x:c r="D11" s="10" t="str">
         <x:v>Use AfC if connected to the subject.</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Do not publish directly to mainspace yet</x:v>
+        <x:v>Treat repeated announcement-style coverage as one source family until proven otherwise.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -764,12 +764,12 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="31" t="str">
-        <x:v>Wikipedia can use primary and affiliated sources to verify limited facts, but they do not establish notability. The current dossier has facts, not yet enough independent profile-depth coverage.</x:v>
-      </x:c>
-      <x:c r="B15" s="31" t="str"/>
-      <x:c r="C15" s="31" t="str"/>
-      <x:c r="D15" s="31" t="str"/>
-      <x:c r="E15" s="31" t="str"/>
+        <x:v>The strongest new material verifies AFRICAST and Headies-related roles, but most of it is project/event coverage rather than independent biographical treatment.</x:v>
+      </x:c>
+      <x:c r="B15" s="31"/>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="31" t="str">
@@ -1805,6 +1805,286 @@
         <x:v>https://en.wikipedia.org/wiki/Wikipedia:Notability_(people)</x:v>
       </x:c>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>F27</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>AFRICAST</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Guardian Nigeria reported that NBC appointed Adeseun Oyeneye, Vice President of Threesixty Africa Group, as Project Coordinator for AFRICAST 2025.</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>2025-09-16</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>S15</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>Use as project-role verification; article is about AFRICAST, not an in-depth biography.</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>https://guardian.ng/features/media/africast-2025-holds-october-20-to-24-in-lagos/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>F28</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>AFRICAST</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>Pulse Nigeria reported that NBC appointed Adeseun Oyeneye as official Project Coordinator for AFRICAST 2025 and described Threesixty Africa Media as project coordination, marketing and sponsorship agency.</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>2025-05-10</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>S16</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>Promotional/event-announcement style; still useful corroboration of role wording.</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>https://www.pulse.ng/story/africast-2025-navigating-the-digital-surge-to-build-a-resilient-african-media-ecosystem-2025051006542969016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>F29</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>AFRICAST</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>Media Rights Agenda reported that Adeseun Oyeneye, Vice-President of Threesixty Africa Group, was appointed official Project Coordinator for AFRICAST 2025.</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>S17</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>Corroborates AFRICAST role; not a biographical feature.</x:v>
+      </x:c>
+      <x:c r="K33" t="str">
+        <x:v>https://mediarightsagenda.org/nbc-unveils-africast-2025-to-drive-digital-innovation-in-african-media/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>F30</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>Headies Mic Check</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>Leadership identified Adeseun Oyeneye as Executive Producer of Headies Mic Check and quoted her on the competition's purpose.</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>2023-08</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>S18</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>Useful for career chronology; watch for syndicated/press-release text overlap.</x:v>
+      </x:c>
+      <x:c r="K34" t="str">
+        <x:v>https://leadership.ng/20-talents-battle-for-n5m-in-airtel-headies-mic-check-competition/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>F31</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Headies Mic Check</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>TeleScope.ng identified Adeseun Oyeneye as Executive Producer of Headies Mic Check and included a quote about the competition's star-development goal.</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>2023-08-28</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>S19</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="J35" t="str">
+        <x:v>Likely corroborative rather than a separate significant source if syndicated.</x:v>
+      </x:c>
+      <x:c r="K35" t="str">
+        <x:v>https://telescope.ng/2023/08/28/headies-mic-check-season-two-airtel-sponsored-competition-elevates-20-talents-to-battle-for-grand-prizes/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>F32</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>Television production</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>Vanguard identified Mrs. Adeseun Oyeneye as content producer of the television show Howfar with Sheila O.</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>2021-07-09</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>S20</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>Secondary</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>Brief mention; useful for chronology only.</x:v>
+      </x:c>
+      <x:c r="K36" t="str">
+        <x:v>https://www.vanguardngr.com/2021/07/sheila-o-premieres-season-3-of-howfar-with-sheila-o/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>F33</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>Video leads</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>YouTube searches found her own channel, a video titled 'Adeseun Oyeneye opens up about working with Mr. Ayo Animashaun,' and 360AFRICATV Mailbox episodes listing Adeseun Oyeneye and Wale Ekundayo as hosts.</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>2026-10-05 search capture</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>S21-S23</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>Lead verified</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>Video/search result</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>Mixed / affiliated</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>Do not use as notability proof; use to guide searches for independent interviews or transcripts.</x:v>
+      </x:c>
+      <x:c r="K37" t="str">
+        <x:v>https://www.youtube.com/results?search_query=%22Adeseun+Oyeneye%22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>F34</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Notability</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>Deeper search found more independent direct mentions and video leads, but the source set still lacks multiple independent sources with substantial biographical treatment.</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>P01, S15-S23</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>Assessment</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>Policy application</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>Mixed</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>Controls readiness</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>This is stronger than the first pass for fact verification, but still not enough for a low-risk standalone mainspace article.</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>https://en.wikipedia.org/wiki/Wikipedia:Notability_(people)</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F5:F200">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Verified"/>
@@ -1812,7 +2092,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bebbf023cc14f4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R106b4c08e050448d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2603,13 +2883,355 @@
         <x:v>Submit draft for review after notability gap is improved.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>S15</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Africast 2025 holds October 20 to 24 in Lagos</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>The Guardian Nigeria</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>2025-09-16</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>https://guardian.ng/features/media/africast-2025-holds-october-20-to-24-in-lagos/</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>News article</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Event coverage with direct role mention</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>Opened in Playwright; direct Adeseun role mention found</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>Verify AFRICAST 2025 appointment as Project Coordinator and VP wording</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>Partial; direct project role but not significant biography coverage</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>Newer Guardian AFRICAST article directly names her; supersedes earlier event-only Guardian lead for this specific role.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>S16</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>AFRICAST 2025: Navigating the Digital Surge to Build a Resilient African Media Ecosystem</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Pulse Nigeria</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>2025-05-10</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>https://www.pulse.ng/story/africast-2025-navigating-the-digital-surge-to-build-a-resilient-african-media-ecosystem-2025051006542969016</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>News article</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Event coverage with direct role mention</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>Opened in Playwright; direct Adeseun role mention found</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>Verify NBC appointment, Threesixty Africa role, and marketing/sponsorship coordination wording</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>Partial; direct project role but not significant biography coverage</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>Text appears promotional/event-announcement style; useful corroboration, not a standalone biographical feature.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>S17</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>NBC Unveils AFRICAST 2025 to Drive Digital Innovation in African Media</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Media Rights Agenda</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>https://mediarightsagenda.org/nbc-unveils-africast-2025-to-drive-digital-innovation-in-african-media/</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>News article</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>Event coverage with direct role mention</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>Opened in Playwright; direct Adeseun role mention found</x:v>
+      </x:c>
+      <x:c r="J25" t="str">
+        <x:v>Corroborate AFRICAST appointment and project-coordination scope</x:v>
+      </x:c>
+      <x:c r="K25" t="str">
+        <x:v>Partial; direct project role but not significant biography coverage</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>Adds a third outlet for the AFRICAST role; article focus remains AFRICAST, not her life/career.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>S18</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>20 Talents Battle For N5m In Airtel Headies Mic Check Competition</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Leadership</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>2023-08</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>https://leadership.ng/20-talents-battle-for-n5m-in-airtel-headies-mic-check-competition/</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>News article</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Project-focused mention with quote</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>Opened in Playwright; direct Adeseun quote found</x:v>
+      </x:c>
+      <x:c r="J26" t="str">
+        <x:v>Verify executive producer role for Headies Mic Check and quote about the competition</x:v>
+      </x:c>
+      <x:c r="K26" t="str">
+        <x:v>Partial; project coverage, not profile-depth</x:v>
+      </x:c>
+      <x:c r="L26" t="str">
+        <x:v>Substantially similar to other Mic Check coverage; treat as corroboration unless editorial independence is confirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>S19</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Headies Mic Check Season Two: Airtel-sponsored competition elevates 20 talents to battle for grand prizes</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>TeleScope.ng</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>2023-08-28</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>https://telescope.ng/2023/08/28/headies-mic-check-season-two-airtel-sponsored-competition-elevates-20-talents-to-battle-for-grand-prizes/</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>News article</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Project-focused mention with quote</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>Opened in Playwright; direct Adeseun role/quote found</x:v>
+      </x:c>
+      <x:c r="J27" t="str">
+        <x:v>Corroborate executive producer role and competition context</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>Partial; project coverage, not profile-depth</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>Text overlaps with other Mic Check reports and may be syndicated or press-release-derived.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>S20</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Sheila O premieres season 3 of “Howfar with Sheila O”</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Vanguard News</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>2021-07-09</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>https://www.vanguardngr.com/2021/07/sheila-o-premieres-season-3-of-howfar-with-sheila-o/</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>News article</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>Independent</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Brief role mention</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>Opened in Playwright; direct Adeseun role mention found</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>Verify content producer role on Howfar with Sheila O</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>Low to partial; brief mention, not biography coverage</x:v>
+      </x:c>
+      <x:c r="L28" t="str">
+        <x:v>Useful for chronology and production credits; not enough as notability proof.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>S21</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>YouTube search result: “Adeseun Oyeneye”</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>YouTube</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>2026-10-05 capture</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>https://www.youtube.com/results?search_query=%22Adeseun+Oyeneye%22</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>Video search result</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>Mixed / platform</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Video leads and channel discovery</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>Opened in Playwright; snapshot saved under .tmp/playwright_youtube_adeseun.yml</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>Lead list for own channel, Ayo Animashaun video, and 360AFRICATV Mailbox episodes</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>Lead only</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>Search result showed her own channel and videos; evaluate each video individually before relying on it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>Adeseun Oyeneye opens up about working with Mr. Ayo Animashaun</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>YouTube / Adeseun Oyeneye channel</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>https://www.youtube.com/watch?v=797xAO4TMg8</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>Video</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>Self-published</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Short first-person / owned-channel video lead</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>Opened in Playwright; page title captured; video result appeared in YouTube search</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>Potential lead for relationship to Ayo Animashaun and Headies/Smooth Promotions career context</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>None for notability unless independently covered</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>Could be useful for leads, but Wikipedia should prefer independent published interviews/transcripts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>S23</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Mailbox episodes hosted by Adeseun Oyeneye and Wale Ekundayo</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>YouTube / 360AFRICATV</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>c. 2024</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>https://www.youtube.com/results?search_query=%22Adeseun+Oyeneye%22+%22360AFRICATV%22</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>Video search result</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Affiliated / owned channel</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Program-hosting video leads</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>Opened in Playwright; search results showed episodes 38, 39, and 41 with host description</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>Verify that she hosted 360AFRICATV Mailbox episodes</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>Low; affiliated/owned-channel evidence</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>Good chronology lead. Need independent reviews or media coverage for Wikipedia weight.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="K5:K100">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Low"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a9a55f45fd446b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bc6329370df4cc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +3607,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb03228192637481a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree8b03f92eeb4f8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3213,7 +3835,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77b3d02a8de24811"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c7e611817e949c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3303,10 +3925,10 @@
         <x:v>Wikipedia needs significant coverage in multiple independent secondary sources.</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Most sources are primary, affiliated, retail metadata, or project mentions.</x:v>
+        <x:v>Added S15-S20 independent direct mentions plus S21-S23 YouTube/video leads; most are project/event mentions or affiliated videos.</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Find 2-3 independent profiles/interviews/features that cover her career in depth.</x:v>
+        <x:v>Find 2-3 independent profiles/interviews/features that cover her career in depth, not only project announcements.</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
         <x:v>Research</x:v>
@@ -3407,10 +4029,10 @@
         <x:v>AFRICAST claims are prominent on the site but not yet directly confirmed in accessible source text.</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Guardian event article does not name her; Radio Now blocked.</x:v>
+        <x:v>Guardian, Pulse and Media Rights Agenda now directly confirm her AFRICAST 2025 Project Coordinator role.</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>Find NBC program, AFRICAST site, press kit, archived Radio Now page, or newspaper PDF naming her.</x:v>
+        <x:v>Find NBC/AFRICAST official program or press kit and assess whether the media reports are original reporting or announcement syndication.</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
         <x:v>Research</x:v>
@@ -3419,7 +4041,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
-        <x:v>Open</x:v>
+        <x:v>Partly closed</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="36" hidden="0" customHeight="1">
@@ -3497,6 +4119,58 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>G09</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Syndication / press-release clustering</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Repeated articles with similar wording may count as one source family rather than multiple independent significant sources.</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>Headies Mic Check and AFRICAST stories repeat role/quote language across several outlets.</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>Identify original reporting, bylined interviews, archive scans, TV transcripts, or features with editorial analysis.</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>G10</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>YouTube/video evidence triage</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Videos can help chronology, but self-published or affiliated channels do not establish Wikipedia notability.</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>YouTube shows own-channel results and 360AFRICATV Mailbox hosting clips.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Search for independent TV/news interviews, podcast transcripts, show notes, and articles reviewing her work.</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
         <x:v>Open</x:v>
       </x:c>
     </x:row>
@@ -3506,7 +4180,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R376ed221f5ca4b51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49584490e9ca408b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3674,7 +4348,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde3a2f3ca7a44941"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cabe2ce11784039"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>